<commit_message>
BOM Review completed CAT24C256WI-GT3 is part ka link or price change hui ha BOM me
</commit_message>
<xml_diff>
--- a/Deliverables/Control_Board/BOM/LCSC_CB_ 500.xlsx
+++ b/Deliverables/Control_Board/BOM/LCSC_CB_ 500.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24527"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\ChrisitanRaun-AnnanasMotor\Deliverables\Control_Board\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\ChrisitanRaun-AnnanasMotor\Deliverables\Control_Board\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA4F8C8D-C86F-4889-B897-9ACF018CD051}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -409,9 +408,6 @@
     <t>onsemi</t>
   </si>
   <si>
-    <t>C79987</t>
-  </si>
-  <si>
     <t>MAGNETIC ANGLE SENSOR</t>
   </si>
   <si>
@@ -620,12 +616,15 @@
   </si>
   <si>
     <t>Out of stock on custom supplier. Alternate added</t>
+  </si>
+  <si>
+    <t>Chipmall</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00000"/>
@@ -1329,7 +1328,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="150">
+  <cellXfs count="153">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1621,40 +1620,10 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -1668,95 +1637,134 @@
     <xf numFmtId="0" fontId="9" fillId="7" borderId="29" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="14" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="29" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="14" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="1" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="16" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="29" xfId="1" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2033,7 +2041,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Y46"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
@@ -2047,8 +2055,8 @@
     <col min="8" max="8" width="14.42578125" style="2" customWidth="1"/>
     <col min="9" max="9" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="6.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.7109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="20.28515625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="18.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="21.85546875" style="1" customWidth="1"/>
     <col min="14" max="14" width="14.140625" style="1" customWidth="1"/>
     <col min="15" max="15" width="17.42578125" style="1" customWidth="1"/>
@@ -2057,38 +2065,38 @@
     <col min="18" max="18" width="13.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="16.42578125" style="1" customWidth="1"/>
     <col min="20" max="22" width="17.7109375" style="1" customWidth="1"/>
-    <col min="23" max="23" width="31.42578125" style="1" customWidth="1"/>
+    <col min="23" max="23" width="28.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="49.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="25" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="16.5" thickBot="1">
-      <c r="A1" s="99" t="s">
-        <v>166</v>
-      </c>
-      <c r="B1" s="100"/>
-      <c r="C1" s="100"/>
-      <c r="D1" s="100"/>
-      <c r="E1" s="100"/>
-      <c r="F1" s="100"/>
-      <c r="G1" s="100"/>
-      <c r="H1" s="100"/>
-      <c r="I1" s="100"/>
-      <c r="J1" s="100"/>
-      <c r="K1" s="100"/>
-      <c r="L1" s="100"/>
-      <c r="M1" s="100"/>
-      <c r="N1" s="100"/>
-      <c r="O1" s="100"/>
-      <c r="P1" s="100"/>
-      <c r="Q1" s="100"/>
-      <c r="R1" s="100"/>
-      <c r="S1" s="100"/>
-      <c r="T1" s="100"/>
-      <c r="U1" s="100"/>
-      <c r="V1" s="100"/>
-      <c r="W1" s="100"/>
-      <c r="X1" s="101"/>
+      <c r="A1" s="138" t="s">
+        <v>165</v>
+      </c>
+      <c r="B1" s="139"/>
+      <c r="C1" s="139"/>
+      <c r="D1" s="139"/>
+      <c r="E1" s="139"/>
+      <c r="F1" s="139"/>
+      <c r="G1" s="139"/>
+      <c r="H1" s="139"/>
+      <c r="I1" s="139"/>
+      <c r="J1" s="139"/>
+      <c r="K1" s="139"/>
+      <c r="L1" s="139"/>
+      <c r="M1" s="139"/>
+      <c r="N1" s="139"/>
+      <c r="O1" s="139"/>
+      <c r="P1" s="139"/>
+      <c r="Q1" s="139"/>
+      <c r="R1" s="139"/>
+      <c r="S1" s="139"/>
+      <c r="T1" s="139"/>
+      <c r="U1" s="139"/>
+      <c r="V1" s="139"/>
+      <c r="W1" s="139"/>
+      <c r="X1" s="140"/>
     </row>
     <row r="2" spans="1:25" ht="16.5" thickBot="1">
       <c r="A2" s="3" t="s">
@@ -2122,19 +2130,19 @@
         <v>9</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="L2" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="M2" s="5" t="s">
         <v>10</v>
       </c>
       <c r="N2" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="O2" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="P2" s="12" t="s">
         <v>11</v>
@@ -2143,19 +2151,19 @@
         <v>12</v>
       </c>
       <c r="R2" s="18" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="S2" s="18" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="T2" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="U2" s="18" t="s">
         <v>185</v>
       </c>
-      <c r="U2" s="18" t="s">
+      <c r="V2" s="5" t="s">
         <v>186</v>
-      </c>
-      <c r="V2" s="5" t="s">
-        <v>187</v>
       </c>
       <c r="W2" s="5" t="s">
         <v>13</v>
@@ -2168,7 +2176,7 @@
       <c r="A3" s="6">
         <v>1</v>
       </c>
-      <c r="B3" s="102" t="s">
+      <c r="B3" s="145" t="s">
         <v>15</v>
       </c>
       <c r="C3" s="29" t="s">
@@ -2204,11 +2212,11 @@
       <c r="M3" s="33">
         <v>4</v>
       </c>
-      <c r="N3" s="33">
+      <c r="N3" s="106">
         <f>M3*500</f>
         <v>2000</v>
       </c>
-      <c r="O3" s="33">
+      <c r="O3" s="106">
         <f>M3*1000</f>
         <v>4000</v>
       </c>
@@ -2226,13 +2234,13 @@
         <v>6.8199999999999997E-2</v>
       </c>
       <c r="T3" s="36">
-        <f>S3*L3</f>
+        <f t="shared" ref="T3:T25" si="0">S3*L3</f>
         <v>139.81</v>
       </c>
       <c r="U3" s="35">
         <v>6.8199999999999997E-2</v>
       </c>
-      <c r="V3" s="36">
+      <c r="V3" s="151">
         <f>U3*K3</f>
         <v>276.20999999999998</v>
       </c>
@@ -2243,12 +2251,12 @@
       <c r="A4" s="6">
         <v>2</v>
       </c>
-      <c r="B4" s="103"/>
+      <c r="B4" s="146"/>
       <c r="C4" s="38" t="s">
         <v>25</v>
       </c>
       <c r="D4" s="90" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E4" s="22" t="s">
         <v>26</v>
@@ -2277,36 +2285,36 @@
       <c r="M4" s="41">
         <v>24</v>
       </c>
-      <c r="N4" s="33">
+      <c r="N4" s="41">
         <f>M4*500</f>
         <v>12000</v>
       </c>
-      <c r="O4" s="33">
-        <f t="shared" ref="O4:O29" si="0">M4*1000</f>
+      <c r="O4" s="41">
+        <f t="shared" ref="O4:O29" si="1">M4*1000</f>
         <v>24000</v>
       </c>
       <c r="P4" s="42" t="s">
         <v>24</v>
       </c>
       <c r="Q4" s="43">
-        <v>4.7000000000000002E-3</v>
+        <v>7.9000000000000008E-3</v>
       </c>
       <c r="R4" s="43">
-        <f t="shared" ref="R4:R27" si="1">Q4*M4</f>
-        <v>0.11280000000000001</v>
+        <f t="shared" ref="R4:R27" si="2">Q4*M4</f>
+        <v>0.18960000000000002</v>
       </c>
       <c r="S4" s="43">
         <v>5.1000000000000004E-3</v>
       </c>
       <c r="T4" s="44">
-        <f>S4*L4</f>
+        <f t="shared" si="0"/>
         <v>61.455000000000005</v>
       </c>
       <c r="U4" s="43">
         <v>5.1000000000000004E-3</v>
       </c>
-      <c r="V4" s="36">
-        <f t="shared" ref="V4:V26" si="2">U4*K4</f>
+      <c r="V4" s="44">
+        <f t="shared" ref="V4:V26" si="3">U4*K4</f>
         <v>122.65500000000002</v>
       </c>
       <c r="W4" s="41"/>
@@ -2316,7 +2324,7 @@
       <c r="A5" s="6">
         <v>3</v>
       </c>
-      <c r="B5" s="103"/>
+      <c r="B5" s="146"/>
       <c r="C5" s="38" t="s">
         <v>31</v>
       </c>
@@ -2350,36 +2358,36 @@
       <c r="M5" s="41">
         <v>1</v>
       </c>
-      <c r="N5" s="33">
-        <f t="shared" ref="N5:N29" si="3">M5*500</f>
+      <c r="N5" s="41">
+        <f t="shared" ref="N5:N29" si="4">M5*500</f>
         <v>500</v>
       </c>
-      <c r="O5" s="33">
-        <f t="shared" si="0"/>
+      <c r="O5" s="41">
+        <f t="shared" si="1"/>
         <v>1000</v>
       </c>
       <c r="P5" s="42" t="s">
         <v>24</v>
       </c>
       <c r="Q5" s="43">
-        <v>0.12640000000000001</v>
+        <v>0.1052</v>
       </c>
       <c r="R5" s="43">
-        <f t="shared" si="1"/>
-        <v>0.12640000000000001</v>
+        <f t="shared" si="2"/>
+        <v>0.1052</v>
       </c>
       <c r="S5" s="43">
         <v>6.7000000000000004E-2</v>
       </c>
       <c r="T5" s="44">
-        <f>S5*L5</f>
+        <f t="shared" si="0"/>
         <v>36.85</v>
       </c>
       <c r="U5" s="43">
         <v>6.7000000000000004E-2</v>
       </c>
-      <c r="V5" s="36">
-        <f t="shared" si="2"/>
+      <c r="V5" s="44">
+        <f t="shared" si="3"/>
         <v>70.350000000000009</v>
       </c>
       <c r="W5" s="41"/>
@@ -2390,7 +2398,7 @@
       <c r="A6" s="6">
         <v>4</v>
       </c>
-      <c r="B6" s="103"/>
+      <c r="B6" s="146"/>
       <c r="C6" s="38" t="s">
         <v>37</v>
       </c>
@@ -2424,12 +2432,12 @@
       <c r="M6" s="41">
         <v>3</v>
       </c>
-      <c r="N6" s="33">
-        <f t="shared" si="3"/>
+      <c r="N6" s="41">
+        <f t="shared" si="4"/>
         <v>1500</v>
       </c>
-      <c r="O6" s="33">
-        <f t="shared" si="0"/>
+      <c r="O6" s="41">
+        <f t="shared" si="1"/>
         <v>3000</v>
       </c>
       <c r="P6" s="19" t="s">
@@ -2439,21 +2447,21 @@
         <v>3.4700000000000002E-2</v>
       </c>
       <c r="R6" s="43">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.1041</v>
       </c>
       <c r="S6" s="43">
         <v>2.1600000000000001E-2</v>
       </c>
       <c r="T6" s="44">
-        <f>S6*L6</f>
+        <f t="shared" si="0"/>
         <v>33.480000000000004</v>
       </c>
       <c r="U6" s="43">
         <v>2.1600000000000001E-2</v>
       </c>
-      <c r="V6" s="36">
-        <f t="shared" si="2"/>
+      <c r="V6" s="44">
+        <f t="shared" si="3"/>
         <v>65.88000000000001</v>
       </c>
       <c r="W6" s="41"/>
@@ -2464,7 +2472,7 @@
       <c r="A7" s="6">
         <v>5</v>
       </c>
-      <c r="B7" s="104"/>
+      <c r="B7" s="147"/>
       <c r="C7" s="48" t="s">
         <v>44</v>
       </c>
@@ -2498,36 +2506,36 @@
       <c r="M7" s="53">
         <v>4</v>
       </c>
-      <c r="N7" s="33">
-        <f t="shared" si="3"/>
+      <c r="N7" s="150">
+        <f t="shared" si="4"/>
         <v>2000</v>
       </c>
-      <c r="O7" s="33">
-        <f t="shared" si="0"/>
+      <c r="O7" s="150">
+        <f t="shared" si="1"/>
         <v>4000</v>
       </c>
       <c r="P7" s="54" t="s">
         <v>24</v>
       </c>
       <c r="Q7" s="55">
-        <v>3.0000000000000001E-3</v>
+        <v>2.5000000000000001E-3</v>
       </c>
       <c r="R7" s="56">
-        <f t="shared" si="1"/>
-        <v>1.2E-2</v>
+        <f t="shared" si="2"/>
+        <v>0.01</v>
       </c>
       <c r="S7" s="56">
         <v>1.9E-3</v>
       </c>
       <c r="T7" s="57">
-        <f>S7*L7</f>
+        <f t="shared" si="0"/>
         <v>3.99</v>
       </c>
       <c r="U7" s="56">
         <v>1.8E-3</v>
       </c>
-      <c r="V7" s="36">
-        <f t="shared" si="2"/>
+      <c r="V7" s="152">
+        <f t="shared" si="3"/>
         <v>7.38</v>
       </c>
       <c r="W7" s="27"/>
@@ -2575,35 +2583,35 @@
         <v>3</v>
       </c>
       <c r="N8" s="33">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1500</v>
       </c>
       <c r="O8" s="33">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>3000</v>
       </c>
       <c r="P8" s="66" t="s">
         <v>24</v>
       </c>
       <c r="Q8" s="67">
-        <v>6.5500000000000003E-2</v>
+        <v>6.8099999999999994E-2</v>
       </c>
       <c r="R8" s="67">
-        <f t="shared" si="1"/>
-        <v>0.19650000000000001</v>
+        <f t="shared" si="2"/>
+        <v>0.20429999999999998</v>
       </c>
       <c r="S8" s="67">
         <v>4.5699999999999998E-2</v>
       </c>
       <c r="T8" s="68">
-        <f>S8*L8</f>
+        <f t="shared" si="0"/>
         <v>70.834999999999994</v>
       </c>
       <c r="U8" s="67">
         <v>4.5699999999999998E-2</v>
       </c>
       <c r="V8" s="36">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>139.38499999999999</v>
       </c>
       <c r="W8" s="65"/>
@@ -2614,7 +2622,7 @@
       <c r="A9" s="6">
         <v>7</v>
       </c>
-      <c r="B9" s="102" t="s">
+      <c r="B9" s="145" t="s">
         <v>59</v>
       </c>
       <c r="C9" s="29" t="s">
@@ -2651,35 +2659,35 @@
         <v>5</v>
       </c>
       <c r="N9" s="33">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2500</v>
       </c>
       <c r="O9" s="33">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>5000</v>
       </c>
       <c r="P9" s="34" t="s">
         <v>24</v>
       </c>
       <c r="Q9" s="35">
-        <v>6.8999999999999999E-3</v>
+        <v>7.0000000000000001E-3</v>
       </c>
       <c r="R9" s="35">
-        <f t="shared" si="1"/>
-        <v>3.4500000000000003E-2</v>
+        <f t="shared" si="2"/>
+        <v>3.5000000000000003E-2</v>
       </c>
       <c r="S9" s="35">
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="T9" s="36">
-        <f>S9*L9</f>
+        <f t="shared" si="0"/>
         <v>12.75</v>
       </c>
       <c r="U9" s="35">
         <v>4.7000000000000002E-3</v>
       </c>
       <c r="V9" s="36">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>23.734999999999999</v>
       </c>
       <c r="W9" s="33"/>
@@ -2690,7 +2698,7 @@
       <c r="A10" s="6">
         <v>8</v>
       </c>
-      <c r="B10" s="104"/>
+      <c r="B10" s="147"/>
       <c r="C10" s="48" t="s">
         <v>66</v>
       </c>
@@ -2725,36 +2733,36 @@
         <v>1</v>
       </c>
       <c r="N10" s="33">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>500</v>
       </c>
       <c r="O10" s="33">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1000</v>
       </c>
       <c r="P10" s="73" t="s">
         <v>24</v>
       </c>
       <c r="Q10" s="56">
-        <v>4.9599999999999998E-2</v>
+        <v>4.58E-2</v>
       </c>
       <c r="R10" s="56">
-        <f t="shared" si="1"/>
-        <v>4.9599999999999998E-2</v>
+        <f t="shared" si="2"/>
+        <v>4.58E-2</v>
       </c>
       <c r="S10" s="56">
-        <v>5.3E-3</v>
+        <v>3.4099999999999998E-2</v>
       </c>
       <c r="T10" s="57">
-        <f>S10*L10</f>
-        <v>2.915</v>
+        <f t="shared" si="0"/>
+        <v>18.754999999999999</v>
       </c>
       <c r="U10" s="56">
-        <v>5.3E-3</v>
+        <v>3.2199999999999999E-2</v>
       </c>
       <c r="V10" s="36">
-        <f t="shared" si="2"/>
-        <v>5.5650000000000004</v>
+        <f t="shared" si="3"/>
+        <v>33.81</v>
       </c>
       <c r="W10" s="53"/>
       <c r="X10" s="58"/>
@@ -2764,7 +2772,7 @@
       <c r="A11" s="6">
         <v>9</v>
       </c>
-      <c r="B11" s="102" t="s">
+      <c r="B11" s="145" t="s">
         <v>72</v>
       </c>
       <c r="C11" s="29" t="s">
@@ -2800,12 +2808,12 @@
       <c r="M11" s="33">
         <v>12</v>
       </c>
-      <c r="N11" s="33">
-        <f t="shared" si="3"/>
+      <c r="N11" s="106">
+        <f t="shared" si="4"/>
         <v>6000</v>
       </c>
-      <c r="O11" s="33">
-        <f t="shared" si="0"/>
+      <c r="O11" s="106">
+        <f t="shared" si="1"/>
         <v>12000</v>
       </c>
       <c r="P11" s="26" t="s">
@@ -2815,21 +2823,21 @@
         <v>1.4E-3</v>
       </c>
       <c r="R11" s="35">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.6799999999999999E-2</v>
       </c>
       <c r="S11" s="35">
         <v>1E-3</v>
       </c>
       <c r="T11" s="36">
-        <f>S11*L11</f>
+        <f t="shared" si="0"/>
         <v>6.1000000000000005</v>
       </c>
       <c r="U11" s="35">
         <v>8.9999999999999998E-4</v>
       </c>
-      <c r="V11" s="36">
-        <f t="shared" si="2"/>
+      <c r="V11" s="151">
+        <f t="shared" si="3"/>
         <v>10.89</v>
       </c>
       <c r="W11" s="33"/>
@@ -2840,7 +2848,7 @@
       <c r="A12" s="6">
         <v>10</v>
       </c>
-      <c r="B12" s="103"/>
+      <c r="B12" s="146"/>
       <c r="C12" s="38" t="s">
         <v>79</v>
       </c>
@@ -2874,12 +2882,12 @@
       <c r="M12" s="41">
         <v>3</v>
       </c>
-      <c r="N12" s="33">
-        <f t="shared" si="3"/>
+      <c r="N12" s="41">
+        <f t="shared" si="4"/>
         <v>1500</v>
       </c>
-      <c r="O12" s="33">
-        <f t="shared" si="0"/>
+      <c r="O12" s="41">
+        <f t="shared" si="1"/>
         <v>3000</v>
       </c>
       <c r="P12" s="19" t="s">
@@ -2889,21 +2897,21 @@
         <v>1.4E-3</v>
       </c>
       <c r="R12" s="43">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4.1999999999999997E-3</v>
       </c>
       <c r="S12" s="43">
         <v>1E-3</v>
       </c>
       <c r="T12" s="44">
-        <f>S12*L12</f>
+        <f t="shared" si="0"/>
         <v>1.6</v>
       </c>
       <c r="U12" s="43">
         <v>8.9999999999999998E-4</v>
       </c>
-      <c r="V12" s="36">
-        <f t="shared" si="2"/>
+      <c r="V12" s="44">
+        <f t="shared" si="3"/>
         <v>2.79</v>
       </c>
       <c r="W12" s="41"/>
@@ -2914,7 +2922,7 @@
       <c r="A13" s="6">
         <v>11</v>
       </c>
-      <c r="B13" s="103"/>
+      <c r="B13" s="146"/>
       <c r="C13" s="38" t="s">
         <v>84</v>
       </c>
@@ -2948,12 +2956,12 @@
       <c r="M13" s="41">
         <v>1</v>
       </c>
-      <c r="N13" s="33">
-        <f t="shared" si="3"/>
+      <c r="N13" s="41">
+        <f t="shared" si="4"/>
         <v>500</v>
       </c>
-      <c r="O13" s="33">
-        <f t="shared" si="0"/>
+      <c r="O13" s="41">
+        <f t="shared" si="1"/>
         <v>1000</v>
       </c>
       <c r="P13" s="76" t="s">
@@ -2963,21 +2971,21 @@
         <v>1.4E-3</v>
       </c>
       <c r="R13" s="43">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.4E-3</v>
       </c>
       <c r="S13" s="43">
         <v>1.4E-3</v>
       </c>
       <c r="T13" s="44">
-        <f>S13*L13</f>
+        <f t="shared" si="0"/>
         <v>0.84</v>
       </c>
       <c r="U13" s="43">
         <v>1.1000000000000001E-3</v>
       </c>
-      <c r="V13" s="36">
-        <f t="shared" si="2"/>
+      <c r="V13" s="44">
+        <f t="shared" si="3"/>
         <v>1.21</v>
       </c>
       <c r="W13" s="75"/>
@@ -2988,7 +2996,7 @@
       <c r="A14" s="6">
         <v>12</v>
       </c>
-      <c r="B14" s="103"/>
+      <c r="B14" s="146"/>
       <c r="C14" s="38" t="s">
         <v>89</v>
       </c>
@@ -3022,36 +3030,36 @@
       <c r="M14" s="41">
         <v>4</v>
       </c>
-      <c r="N14" s="33">
-        <f t="shared" si="3"/>
+      <c r="N14" s="41">
+        <f t="shared" si="4"/>
         <v>2000</v>
       </c>
-      <c r="O14" s="33">
-        <f t="shared" si="0"/>
+      <c r="O14" s="41">
+        <f t="shared" si="1"/>
         <v>4000</v>
       </c>
       <c r="P14" s="19" t="s">
         <v>24</v>
       </c>
       <c r="Q14" s="43">
-        <v>1.4E-3</v>
+        <v>1.1999999999999999E-3</v>
       </c>
       <c r="R14" s="43">
-        <f t="shared" si="1"/>
-        <v>5.5999999999999999E-3</v>
+        <f t="shared" si="2"/>
+        <v>4.7999999999999996E-3</v>
       </c>
       <c r="S14" s="43">
         <v>8.9999999999999998E-4</v>
       </c>
       <c r="T14" s="44">
-        <f>S14*L14</f>
+        <f t="shared" si="0"/>
         <v>1.89</v>
       </c>
       <c r="U14" s="43">
         <v>8.9999999999999998E-4</v>
       </c>
-      <c r="V14" s="36">
-        <f t="shared" si="2"/>
+      <c r="V14" s="44">
+        <f t="shared" si="3"/>
         <v>3.69</v>
       </c>
       <c r="W14" s="41"/>
@@ -3062,7 +3070,7 @@
       <c r="A15" s="6">
         <v>13</v>
       </c>
-      <c r="B15" s="105"/>
+      <c r="B15" s="148"/>
       <c r="C15" s="92" t="s">
         <v>94</v>
       </c>
@@ -3096,36 +3104,36 @@
       <c r="M15" s="93">
         <v>2</v>
       </c>
-      <c r="N15" s="33">
-        <f t="shared" si="3"/>
+      <c r="N15" s="41">
+        <f t="shared" si="4"/>
         <v>1000</v>
       </c>
-      <c r="O15" s="33">
-        <f t="shared" si="0"/>
+      <c r="O15" s="41">
+        <f t="shared" si="1"/>
         <v>2000</v>
       </c>
       <c r="P15" s="94" t="s">
         <v>24</v>
       </c>
       <c r="Q15" s="43">
-        <v>1.5E-3</v>
+        <v>1.1999999999999999E-3</v>
       </c>
       <c r="R15" s="43">
-        <f t="shared" si="1"/>
-        <v>3.0000000000000001E-3</v>
+        <f t="shared" si="2"/>
+        <v>2.3999999999999998E-3</v>
       </c>
       <c r="S15" s="43">
         <v>8.9999999999999998E-4</v>
       </c>
       <c r="T15" s="44">
-        <f>S15*L15</f>
+        <f t="shared" si="0"/>
         <v>0.99</v>
       </c>
       <c r="U15" s="43">
         <v>8.9999999999999998E-4</v>
       </c>
-      <c r="V15" s="36">
-        <f t="shared" si="2"/>
+      <c r="V15" s="44">
+        <f t="shared" si="3"/>
         <v>1.89</v>
       </c>
       <c r="W15" s="41"/>
@@ -3136,7 +3144,7 @@
       <c r="A16" s="6">
         <v>14</v>
       </c>
-      <c r="B16" s="105"/>
+      <c r="B16" s="148"/>
       <c r="C16" s="92" t="s">
         <v>99</v>
       </c>
@@ -3170,36 +3178,36 @@
       <c r="M16" s="93">
         <v>1</v>
       </c>
-      <c r="N16" s="33">
-        <f t="shared" si="3"/>
+      <c r="N16" s="41">
+        <f t="shared" si="4"/>
         <v>500</v>
       </c>
-      <c r="O16" s="33">
-        <f t="shared" si="0"/>
+      <c r="O16" s="41">
+        <f t="shared" si="1"/>
         <v>1000</v>
       </c>
       <c r="P16" s="94" t="s">
         <v>24</v>
       </c>
       <c r="Q16" s="43">
-        <v>1.6000000000000001E-3</v>
+        <v>1.5E-3</v>
       </c>
       <c r="R16" s="43">
-        <f t="shared" si="1"/>
-        <v>1.6000000000000001E-3</v>
+        <f t="shared" si="2"/>
+        <v>1.5E-3</v>
       </c>
       <c r="S16" s="43">
         <v>1.5E-3</v>
       </c>
       <c r="T16" s="44">
-        <f>S16*L16</f>
+        <f t="shared" si="0"/>
         <v>0.9</v>
       </c>
       <c r="U16" s="43">
         <v>1.1999999999999999E-3</v>
       </c>
-      <c r="V16" s="36">
-        <f t="shared" si="2"/>
+      <c r="V16" s="44">
+        <f t="shared" si="3"/>
         <v>1.3199999999999998</v>
       </c>
       <c r="W16" s="41"/>
@@ -3210,7 +3218,7 @@
       <c r="A17" s="6">
         <v>15</v>
       </c>
-      <c r="B17" s="104"/>
+      <c r="B17" s="147"/>
       <c r="C17" s="48" t="s">
         <v>104</v>
       </c>
@@ -3244,36 +3252,36 @@
       <c r="M17" s="53">
         <v>1</v>
       </c>
-      <c r="N17" s="33">
-        <f t="shared" si="3"/>
+      <c r="N17" s="150">
+        <f t="shared" si="4"/>
         <v>500</v>
       </c>
-      <c r="O17" s="33">
-        <f t="shared" si="0"/>
+      <c r="O17" s="150">
+        <f t="shared" si="1"/>
         <v>1000</v>
       </c>
       <c r="P17" s="54" t="s">
         <v>24</v>
       </c>
       <c r="Q17" s="56">
-        <v>1.6799999999999999E-2</v>
+        <v>1.37E-2</v>
       </c>
       <c r="R17" s="56">
-        <f t="shared" si="1"/>
-        <v>1.6799999999999999E-2</v>
+        <f t="shared" si="2"/>
+        <v>1.37E-2</v>
       </c>
       <c r="S17" s="56">
         <v>1.06E-2</v>
       </c>
       <c r="T17" s="57">
-        <f>S17*L17</f>
+        <f t="shared" si="0"/>
         <v>5.7240000000000002</v>
       </c>
       <c r="U17" s="56">
         <v>0.01</v>
       </c>
-      <c r="V17" s="36">
-        <f t="shared" si="2"/>
+      <c r="V17" s="152">
+        <f t="shared" si="3"/>
         <v>10.4</v>
       </c>
       <c r="W17" s="53"/>
@@ -3321,35 +3329,35 @@
         <v>1</v>
       </c>
       <c r="N18" s="33">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>500</v>
       </c>
       <c r="O18" s="33">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1000</v>
       </c>
       <c r="P18" s="66" t="s">
         <v>24</v>
       </c>
       <c r="Q18" s="67">
-        <v>7.2700000000000001E-2</v>
+        <v>8.5500000000000007E-2</v>
       </c>
       <c r="R18" s="67">
-        <f t="shared" si="1"/>
-        <v>7.2700000000000001E-2</v>
+        <f t="shared" si="2"/>
+        <v>8.5500000000000007E-2</v>
       </c>
       <c r="S18" s="67">
         <v>4.8099999999999997E-2</v>
       </c>
       <c r="T18" s="68">
-        <f>S18*L18</f>
+        <f t="shared" si="0"/>
         <v>26.454999999999998</v>
       </c>
       <c r="U18" s="67">
         <v>4.8099999999999997E-2</v>
       </c>
       <c r="V18" s="36">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>50.504999999999995</v>
       </c>
       <c r="W18" s="65"/>
@@ -3360,7 +3368,7 @@
       <c r="A19" s="6">
         <v>17</v>
       </c>
-      <c r="B19" s="102" t="s">
+      <c r="B19" s="145" t="s">
         <v>116</v>
       </c>
       <c r="C19" s="29" t="s">
@@ -3370,19 +3378,19 @@
         <v>118</v>
       </c>
       <c r="E19" s="33" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F19" s="21" t="s">
         <v>119</v>
       </c>
       <c r="G19" s="71" t="s">
+        <v>167</v>
+      </c>
+      <c r="H19" s="30" t="s">
+        <v>162</v>
+      </c>
+      <c r="I19" s="30" t="s">
         <v>168</v>
-      </c>
-      <c r="H19" s="30" t="s">
-        <v>163</v>
-      </c>
-      <c r="I19" s="30" t="s">
-        <v>169</v>
       </c>
       <c r="J19" s="30" t="s">
         <v>58</v>
@@ -3396,36 +3404,36 @@
       <c r="M19" s="95">
         <v>1</v>
       </c>
-      <c r="N19" s="33">
+      <c r="N19" s="106">
+        <f t="shared" si="4"/>
+        <v>500</v>
+      </c>
+      <c r="O19" s="106">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+      <c r="P19" s="118" t="s">
+        <v>142</v>
+      </c>
+      <c r="Q19" s="119">
+        <v>21.26</v>
+      </c>
+      <c r="R19" s="35">
+        <f t="shared" si="2"/>
+        <v>21.26</v>
+      </c>
+      <c r="S19" s="119">
+        <v>21.26</v>
+      </c>
+      <c r="T19" s="36">
+        <f t="shared" si="0"/>
+        <v>10842.6</v>
+      </c>
+      <c r="U19" s="119">
+        <v>21.26</v>
+      </c>
+      <c r="V19" s="151">
         <f t="shared" si="3"/>
-        <v>500</v>
-      </c>
-      <c r="O19" s="33">
-        <f t="shared" si="0"/>
-        <v>1000</v>
-      </c>
-      <c r="P19" s="134" t="s">
-        <v>143</v>
-      </c>
-      <c r="Q19" s="135">
-        <v>21.26</v>
-      </c>
-      <c r="R19" s="35">
-        <f t="shared" si="1"/>
-        <v>21.26</v>
-      </c>
-      <c r="S19" s="135">
-        <v>21.26</v>
-      </c>
-      <c r="T19" s="36">
-        <f>S19*L19</f>
-        <v>10842.6</v>
-      </c>
-      <c r="U19" s="135">
-        <v>21.26</v>
-      </c>
-      <c r="V19" s="36">
-        <f t="shared" si="2"/>
         <v>21472.600000000002</v>
       </c>
       <c r="W19" s="33"/>
@@ -3436,7 +3444,7 @@
       <c r="A20" s="6">
         <v>18</v>
       </c>
-      <c r="B20" s="103"/>
+      <c r="B20" s="146"/>
       <c r="C20" s="80" t="s">
         <v>120</v>
       </c>
@@ -3452,8 +3460,8 @@
       <c r="G20" s="23" t="s">
         <v>124</v>
       </c>
-      <c r="H20" s="40" t="s">
-        <v>125</v>
+      <c r="H20" s="39" t="s">
+        <v>22</v>
       </c>
       <c r="I20" s="46" t="s">
         <v>22</v>
@@ -3470,37 +3478,37 @@
       <c r="M20" s="41">
         <v>1</v>
       </c>
-      <c r="N20" s="33">
+      <c r="N20" s="41">
+        <f t="shared" si="4"/>
+        <v>500</v>
+      </c>
+      <c r="O20" s="41">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+      <c r="P20" s="118" t="s">
+        <v>194</v>
+      </c>
+      <c r="Q20" s="43">
+        <v>0.35243799999999997</v>
+      </c>
+      <c r="R20" s="43">
+        <f t="shared" si="2"/>
+        <v>0.35243799999999997</v>
+      </c>
+      <c r="S20" s="43">
+        <v>0.28717100000000001</v>
+      </c>
+      <c r="T20" s="44">
+        <f t="shared" si="0"/>
+        <v>146.45721</v>
+      </c>
+      <c r="U20" s="43">
+        <v>0.28717100000000001</v>
+      </c>
+      <c r="V20" s="44">
         <f t="shared" si="3"/>
-        <v>500</v>
-      </c>
-      <c r="O20" s="33">
-        <f t="shared" si="0"/>
-        <v>1000</v>
-      </c>
-      <c r="P20" s="136" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q20" s="43">
-        <v>0.44</v>
-      </c>
-      <c r="R20" s="43">
-        <f t="shared" si="1"/>
-        <v>0.44</v>
-      </c>
-      <c r="S20" s="43">
-        <v>0.29759999999999998</v>
-      </c>
-      <c r="T20" s="44">
-        <f>S20*L20</f>
-        <v>151.77599999999998</v>
-      </c>
-      <c r="U20" s="43">
-        <v>0.29399999999999998</v>
-      </c>
-      <c r="V20" s="36">
-        <f t="shared" si="2"/>
-        <v>296.94</v>
+        <v>290.04271</v>
       </c>
       <c r="W20" s="41"/>
       <c r="X20" s="45"/>
@@ -3510,21 +3518,21 @@
       <c r="A21" s="6">
         <v>19</v>
       </c>
-      <c r="B21" s="103"/>
+      <c r="B21" s="146"/>
       <c r="C21" s="38" t="s">
+        <v>125</v>
+      </c>
+      <c r="D21" s="22" t="s">
         <v>126</v>
-      </c>
-      <c r="D21" s="22" t="s">
-        <v>127</v>
       </c>
       <c r="E21" s="22" t="s">
         <v>122</v>
       </c>
       <c r="F21" s="22" t="s">
+        <v>127</v>
+      </c>
+      <c r="G21" s="39" t="s">
         <v>128</v>
-      </c>
-      <c r="G21" s="39" t="s">
-        <v>129</v>
       </c>
       <c r="H21" s="39" t="s">
         <v>22</v>
@@ -3538,46 +3546,46 @@
       <c r="K21" s="39">
         <v>1010</v>
       </c>
-      <c r="L21" s="131">
+      <c r="L21" s="115">
         <v>510</v>
       </c>
       <c r="M21" s="96">
         <v>1</v>
       </c>
-      <c r="N21" s="33">
-        <f t="shared" si="3"/>
+      <c r="N21" s="41">
+        <f t="shared" si="4"/>
         <v>500</v>
       </c>
-      <c r="O21" s="33">
-        <f t="shared" si="0"/>
+      <c r="O21" s="41">
+        <f t="shared" si="1"/>
         <v>1000</v>
       </c>
-      <c r="P21" s="136" t="s">
-        <v>148</v>
-      </c>
-      <c r="Q21" s="137">
+      <c r="P21" s="120" t="s">
+        <v>147</v>
+      </c>
+      <c r="Q21" s="121">
         <v>2.7839999999999998</v>
       </c>
       <c r="R21" s="43">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.7839999999999998</v>
       </c>
       <c r="S21" s="43">
         <v>2.7839999999999998</v>
       </c>
       <c r="T21" s="44">
-        <f>S21*L21</f>
+        <f t="shared" si="0"/>
         <v>1419.84</v>
       </c>
       <c r="U21" s="43">
         <v>2.7839999999999998</v>
       </c>
-      <c r="V21" s="36">
-        <f t="shared" si="2"/>
+      <c r="V21" s="44">
+        <f t="shared" si="3"/>
         <v>2811.8399999999997</v>
       </c>
-      <c r="W21" s="138" t="s">
-        <v>161</v>
+      <c r="W21" s="122" t="s">
+        <v>160</v>
       </c>
       <c r="X21" s="45">
         <v>1.1904999999999999</v>
@@ -3588,24 +3596,24 @@
       <c r="A22" s="6">
         <v>20</v>
       </c>
-      <c r="B22" s="104"/>
+      <c r="B22" s="147"/>
       <c r="C22" s="48" t="s">
+        <v>129</v>
+      </c>
+      <c r="D22" s="49" t="s">
         <v>130</v>
       </c>
-      <c r="D22" s="49" t="s">
+      <c r="E22" s="49" t="s">
         <v>131</v>
       </c>
-      <c r="E22" s="49" t="s">
+      <c r="F22" s="49" t="s">
         <v>132</v>
       </c>
-      <c r="F22" s="49" t="s">
+      <c r="G22" s="49" t="s">
         <v>133</v>
       </c>
-      <c r="G22" s="49" t="s">
+      <c r="H22" s="49" t="s">
         <v>134</v>
-      </c>
-      <c r="H22" s="49" t="s">
-        <v>135</v>
       </c>
       <c r="I22" s="49" t="s">
         <v>22</v>
@@ -3622,40 +3630,40 @@
       <c r="M22" s="97">
         <v>1</v>
       </c>
-      <c r="N22" s="33">
-        <f t="shared" si="3"/>
+      <c r="N22" s="150">
+        <f t="shared" si="4"/>
         <v>500</v>
       </c>
-      <c r="O22" s="33">
-        <f t="shared" si="0"/>
+      <c r="O22" s="150">
+        <f t="shared" si="1"/>
         <v>1000</v>
       </c>
-      <c r="P22" s="139" t="s">
-        <v>148</v>
+      <c r="P22" s="123" t="s">
+        <v>147</v>
       </c>
       <c r="Q22" s="56">
         <v>0.4</v>
       </c>
       <c r="R22" s="56">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.4</v>
       </c>
       <c r="S22" s="56">
         <v>0.4</v>
       </c>
       <c r="T22" s="57">
-        <f>S22*L22</f>
+        <f t="shared" si="0"/>
         <v>204</v>
       </c>
       <c r="U22" s="56">
         <v>0.4</v>
       </c>
-      <c r="V22" s="36">
-        <f t="shared" si="2"/>
+      <c r="V22" s="152">
+        <f t="shared" si="3"/>
         <v>404</v>
       </c>
-      <c r="W22" s="140" t="s">
-        <v>161</v>
+      <c r="W22" s="124" t="s">
+        <v>160</v>
       </c>
       <c r="X22" s="58">
         <v>0.79400000000000004</v>
@@ -3666,29 +3674,29 @@
       <c r="A23" s="6">
         <v>21</v>
       </c>
-      <c r="B23" s="102" t="s">
+      <c r="B23" s="145" t="s">
+        <v>135</v>
+      </c>
+      <c r="C23" s="29" t="s">
         <v>136</v>
       </c>
-      <c r="C23" s="29" t="s">
+      <c r="D23" s="21" t="s">
         <v>137</v>
-      </c>
-      <c r="D23" s="21" t="s">
-        <v>138</v>
       </c>
       <c r="E23" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="F23" s="21" t="s">
-        <v>139</v>
+      <c r="F23" s="16" t="s">
+        <v>138</v>
       </c>
       <c r="G23" s="33" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="H23" s="33" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I23" s="71" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="J23" s="71"/>
       <c r="K23" s="71">
@@ -3701,40 +3709,40 @@
         <v>1</v>
       </c>
       <c r="N23" s="33">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>500</v>
       </c>
       <c r="O23" s="33">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1000</v>
       </c>
-      <c r="P23" s="141" t="s">
+      <c r="P23" s="125" t="s">
         <v>24</v>
       </c>
       <c r="Q23" s="35">
         <v>0.1077</v>
       </c>
       <c r="R23" s="35">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.1077</v>
       </c>
       <c r="S23" s="35">
         <v>6.3600000000000004E-2</v>
       </c>
       <c r="T23" s="36">
-        <f>S23*L23</f>
+        <f t="shared" si="0"/>
         <v>33.072000000000003</v>
       </c>
       <c r="U23" s="35">
         <v>6.3600000000000004E-2</v>
       </c>
       <c r="V23" s="36">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>64.872</v>
       </c>
-      <c r="W23" s="142"/>
+      <c r="W23" s="126"/>
       <c r="X23" s="37" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="Y23" s="15"/>
     </row>
@@ -3742,30 +3750,30 @@
       <c r="A24" s="6">
         <v>22</v>
       </c>
-      <c r="B24" s="104"/>
+      <c r="B24" s="147"/>
       <c r="C24" s="48" t="s">
+        <v>139</v>
+      </c>
+      <c r="D24" s="49" t="s">
         <v>140</v>
-      </c>
-      <c r="D24" s="49" t="s">
-        <v>141</v>
       </c>
       <c r="E24" s="49" t="s">
         <v>113</v>
       </c>
       <c r="F24" s="49" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G24" s="49" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="H24" s="49" t="s">
         <v>22</v>
       </c>
       <c r="I24" s="49" t="s">
+        <v>162</v>
+      </c>
+      <c r="J24" s="49" t="s">
         <v>163</v>
-      </c>
-      <c r="J24" s="49" t="s">
-        <v>164</v>
       </c>
       <c r="K24" s="49">
         <v>1020</v>
@@ -3777,38 +3785,38 @@
         <v>1</v>
       </c>
       <c r="N24" s="33">
+        <f t="shared" si="4"/>
+        <v>500</v>
+      </c>
+      <c r="O24" s="33">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+      <c r="P24" s="123" t="s">
+        <v>142</v>
+      </c>
+      <c r="Q24" s="127">
+        <v>0.86619999999999997</v>
+      </c>
+      <c r="R24" s="56">
+        <f t="shared" si="2"/>
+        <v>0.86619999999999997</v>
+      </c>
+      <c r="S24" s="127">
+        <v>0.86619999999999997</v>
+      </c>
+      <c r="T24" s="57">
+        <f t="shared" si="0"/>
+        <v>450.42399999999998</v>
+      </c>
+      <c r="U24" s="127">
+        <v>0.86619999999999997</v>
+      </c>
+      <c r="V24" s="36">
         <f t="shared" si="3"/>
-        <v>500</v>
-      </c>
-      <c r="O24" s="33">
-        <f t="shared" si="0"/>
-        <v>1000</v>
-      </c>
-      <c r="P24" s="139" t="s">
-        <v>143</v>
-      </c>
-      <c r="Q24" s="143">
-        <v>0.86619999999999997</v>
-      </c>
-      <c r="R24" s="56">
-        <f t="shared" si="1"/>
-        <v>0.86619999999999997</v>
-      </c>
-      <c r="S24" s="143">
-        <v>0.86619999999999997</v>
-      </c>
-      <c r="T24" s="57">
-        <f>S24*L24</f>
-        <v>450.42399999999998</v>
-      </c>
-      <c r="U24" s="143">
-        <v>0.86619999999999997</v>
-      </c>
-      <c r="V24" s="36">
-        <f t="shared" si="2"/>
         <v>883.524</v>
       </c>
-      <c r="W24" s="144"/>
+      <c r="W24" s="128"/>
       <c r="X24" s="58"/>
       <c r="Y24" s="15"/>
     </row>
@@ -3816,34 +3824,34 @@
       <c r="A25" s="6">
         <v>23</v>
       </c>
-      <c r="B25" s="106" t="s">
+      <c r="B25" s="149" t="s">
+        <v>143</v>
+      </c>
+      <c r="C25" s="116" t="s">
+        <v>169</v>
+      </c>
+      <c r="D25" s="117" t="s">
+        <v>171</v>
+      </c>
+      <c r="E25" s="117" t="s">
         <v>144</v>
       </c>
-      <c r="C25" s="132" t="s">
-        <v>170</v>
-      </c>
-      <c r="D25" s="133" t="s">
-        <v>172</v>
-      </c>
-      <c r="E25" s="133" t="s">
+      <c r="F25" s="117" t="s">
         <v>145</v>
       </c>
-      <c r="F25" s="133" t="s">
+      <c r="G25" s="117" t="s">
         <v>146</v>
       </c>
-      <c r="G25" s="133" t="s">
-        <v>147</v>
-      </c>
-      <c r="H25" s="133" t="s">
+      <c r="H25" s="117" t="s">
+        <v>162</v>
+      </c>
+      <c r="I25" s="117" t="s">
+        <v>22</v>
+      </c>
+      <c r="J25" s="117" t="s">
         <v>163</v>
       </c>
-      <c r="I25" s="133" t="s">
-        <v>22</v>
-      </c>
-      <c r="J25" s="133" t="s">
-        <v>164</v>
-      </c>
-      <c r="K25" s="133">
+      <c r="K25" s="117">
         <v>140</v>
       </c>
       <c r="L25" s="33">
@@ -3852,16 +3860,16 @@
       <c r="M25" s="95">
         <v>1</v>
       </c>
-      <c r="N25" s="33">
-        <f t="shared" si="3"/>
+      <c r="N25" s="106">
+        <f t="shared" si="4"/>
         <v>500</v>
       </c>
-      <c r="O25" s="33">
-        <f t="shared" si="0"/>
+      <c r="O25" s="106">
+        <f t="shared" si="1"/>
         <v>1000</v>
       </c>
-      <c r="P25" s="134" t="s">
-        <v>148</v>
+      <c r="P25" s="118" t="s">
+        <v>147</v>
       </c>
       <c r="Q25" s="35">
         <v>0.48</v>
@@ -3873,18 +3881,18 @@
         <v>0.48</v>
       </c>
       <c r="T25" s="36">
-        <f>S25*L25</f>
+        <f t="shared" si="0"/>
         <v>33.6</v>
       </c>
       <c r="U25" s="35">
         <v>0.48</v>
       </c>
-      <c r="V25" s="36">
-        <f t="shared" si="2"/>
+      <c r="V25" s="151">
+        <f t="shared" si="3"/>
         <v>67.2</v>
       </c>
-      <c r="W25" s="145" t="s">
-        <v>193</v>
+      <c r="W25" s="129" t="s">
+        <v>192</v>
       </c>
       <c r="X25" s="37"/>
       <c r="Y25" s="15"/>
@@ -3893,32 +3901,32 @@
       <c r="A26" s="6">
         <v>24</v>
       </c>
-      <c r="B26" s="106"/>
+      <c r="B26" s="149"/>
       <c r="C26" s="38" t="s">
-        <v>171</v>
-      </c>
-      <c r="D26" s="133" t="s">
+        <v>170</v>
+      </c>
+      <c r="D26" s="117" t="s">
+        <v>173</v>
+      </c>
+      <c r="E26" s="22" t="s">
+        <v>172</v>
+      </c>
+      <c r="F26" s="22" t="s">
         <v>174</v>
       </c>
-      <c r="E26" s="22" t="s">
-        <v>173</v>
-      </c>
-      <c r="F26" s="22" t="s">
-        <v>175</v>
-      </c>
       <c r="G26" s="22" t="s">
-        <v>147</v>
-      </c>
-      <c r="H26" s="133" t="s">
+        <v>146</v>
+      </c>
+      <c r="H26" s="117" t="s">
+        <v>162</v>
+      </c>
+      <c r="I26" s="117" t="s">
+        <v>168</v>
+      </c>
+      <c r="J26" s="117" t="s">
         <v>163</v>
       </c>
-      <c r="I26" s="133" t="s">
-        <v>169</v>
-      </c>
-      <c r="J26" s="133" t="s">
-        <v>164</v>
-      </c>
-      <c r="K26" s="133">
+      <c r="K26" s="117">
         <v>180</v>
       </c>
       <c r="L26" s="41">
@@ -3928,37 +3936,37 @@
         <v>1</v>
       </c>
       <c r="N26" s="41">
+        <f t="shared" si="4"/>
+        <v>500</v>
+      </c>
+      <c r="O26" s="41">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+      <c r="P26" s="130" t="s">
+        <v>147</v>
+      </c>
+      <c r="Q26" s="131">
+        <v>0.48</v>
+      </c>
+      <c r="R26" s="131">
+        <v>0.48</v>
+      </c>
+      <c r="S26" s="131">
+        <v>0.48</v>
+      </c>
+      <c r="T26" s="132">
+        <f t="shared" ref="T26" si="5">S26*L26</f>
+        <v>43.199999999999996</v>
+      </c>
+      <c r="U26" s="131">
+        <v>0.48</v>
+      </c>
+      <c r="V26" s="44">
         <f t="shared" si="3"/>
-        <v>500</v>
-      </c>
-      <c r="O26" s="33">
-        <f t="shared" si="0"/>
-        <v>1000</v>
-      </c>
-      <c r="P26" s="146" t="s">
-        <v>148</v>
-      </c>
-      <c r="Q26" s="147">
-        <v>0.48</v>
-      </c>
-      <c r="R26" s="147">
-        <v>0.48</v>
-      </c>
-      <c r="S26" s="147">
-        <v>0.48</v>
-      </c>
-      <c r="T26" s="148">
-        <f t="shared" ref="T26" si="4">S26*L26</f>
-        <v>43.199999999999996</v>
-      </c>
-      <c r="U26" s="147">
-        <v>0.48</v>
-      </c>
-      <c r="V26" s="36">
-        <f t="shared" si="2"/>
         <v>86.399999999999991</v>
       </c>
-      <c r="W26" s="149"/>
+      <c r="W26" s="133"/>
       <c r="X26" s="45"/>
       <c r="Y26" s="15"/>
     </row>
@@ -3966,30 +3974,30 @@
       <c r="A27" s="6">
         <v>25</v>
       </c>
-      <c r="B27" s="103"/>
+      <c r="B27" s="146"/>
       <c r="C27" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D27" s="22" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E27" s="22" t="s">
         <v>113</v>
       </c>
       <c r="F27" s="22" t="s">
+        <v>177</v>
+      </c>
+      <c r="G27" s="22" t="s">
         <v>178</v>
       </c>
-      <c r="G27" s="22" t="s">
-        <v>179</v>
-      </c>
       <c r="H27" s="22" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="I27" s="22" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="J27" s="22" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K27" s="22">
         <v>1020</v>
@@ -4000,22 +4008,22 @@
       <c r="M27" s="96">
         <v>1</v>
       </c>
-      <c r="N27" s="33">
-        <f t="shared" si="3"/>
+      <c r="N27" s="41">
+        <f t="shared" si="4"/>
         <v>500</v>
       </c>
-      <c r="O27" s="33">
-        <f t="shared" si="0"/>
+      <c r="O27" s="41">
+        <f t="shared" si="1"/>
         <v>1000</v>
       </c>
-      <c r="P27" s="139" t="s">
-        <v>148</v>
+      <c r="P27" s="123" t="s">
+        <v>147</v>
       </c>
       <c r="Q27" s="43">
         <v>0.45</v>
       </c>
       <c r="R27" s="43">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0.45</v>
       </c>
       <c r="S27" s="43">
@@ -4028,12 +4036,12 @@
       <c r="U27" s="43">
         <v>0.45</v>
       </c>
-      <c r="V27" s="36">
+      <c r="V27" s="152">
         <f>U27*K27</f>
         <v>459</v>
       </c>
       <c r="W27" s="41" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="X27" s="45"/>
       <c r="Y27" s="15"/>
@@ -4042,67 +4050,67 @@
       <c r="A28" s="6">
         <v>26</v>
       </c>
-      <c r="B28" s="103"/>
+      <c r="B28" s="146"/>
       <c r="C28" s="81" t="s">
+        <v>149</v>
+      </c>
+      <c r="D28" s="20" t="s">
         <v>150</v>
       </c>
-      <c r="D28" s="20" t="s">
+      <c r="E28" s="20" t="s">
         <v>151</v>
       </c>
-      <c r="E28" s="20" t="s">
-        <v>152</v>
-      </c>
       <c r="F28" s="82" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G28" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="H28" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="I28" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="J28" s="20" t="s">
         <v>162</v>
       </c>
-      <c r="H28" s="20" t="s">
-        <v>162</v>
-      </c>
-      <c r="I28" s="20" t="s">
-        <v>162</v>
-      </c>
-      <c r="J28" s="20" t="s">
-        <v>163</v>
-      </c>
       <c r="K28" s="20" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L28" s="20" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="M28" s="83">
         <v>5</v>
       </c>
-      <c r="N28" s="33">
-        <f t="shared" si="3"/>
+      <c r="N28" s="41">
+        <f t="shared" si="4"/>
         <v>2500</v>
       </c>
-      <c r="O28" s="33">
-        <f t="shared" si="0"/>
+      <c r="O28" s="41">
+        <f t="shared" si="1"/>
         <v>5000</v>
       </c>
       <c r="P28" s="20" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="Q28" s="20" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="R28" s="20" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="S28" s="20" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="T28" s="20" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="U28" s="20"/>
       <c r="V28" s="20"/>
       <c r="W28" s="84" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="X28" s="85"/>
       <c r="Y28" s="15"/>
@@ -4111,67 +4119,67 @@
       <c r="A29" s="98">
         <v>27</v>
       </c>
-      <c r="B29" s="104"/>
+      <c r="B29" s="147"/>
       <c r="C29" s="86" t="s">
+        <v>153</v>
+      </c>
+      <c r="D29" s="87" t="s">
         <v>154</v>
       </c>
-      <c r="D29" s="87" t="s">
+      <c r="E29" s="28" t="s">
         <v>155</v>
       </c>
-      <c r="E29" s="28" t="s">
-        <v>156</v>
-      </c>
       <c r="F29" s="87" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G29" s="28" t="s">
+        <v>161</v>
+      </c>
+      <c r="H29" s="28" t="s">
+        <v>161</v>
+      </c>
+      <c r="I29" s="28" t="s">
+        <v>161</v>
+      </c>
+      <c r="J29" s="28" t="s">
         <v>162</v>
       </c>
-      <c r="H29" s="28" t="s">
-        <v>162</v>
-      </c>
-      <c r="I29" s="28" t="s">
-        <v>162</v>
-      </c>
-      <c r="J29" s="28" t="s">
-        <v>163</v>
-      </c>
       <c r="K29" s="28" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L29" s="28" t="s">
-        <v>162</v>
-      </c>
-      <c r="M29" s="115">
+        <v>161</v>
+      </c>
+      <c r="M29" s="105">
         <v>3</v>
       </c>
-      <c r="N29" s="116">
-        <f t="shared" si="3"/>
+      <c r="N29" s="65">
+        <f t="shared" si="4"/>
         <v>1500</v>
       </c>
-      <c r="O29" s="116">
-        <f t="shared" si="0"/>
+      <c r="O29" s="65">
+        <f t="shared" si="1"/>
         <v>3000</v>
       </c>
-      <c r="P29" s="117" t="s">
-        <v>162</v>
-      </c>
-      <c r="Q29" s="117" t="s">
-        <v>162</v>
-      </c>
-      <c r="R29" s="117" t="s">
-        <v>162</v>
-      </c>
-      <c r="S29" s="117" t="s">
-        <v>162</v>
-      </c>
-      <c r="T29" s="117" t="s">
-        <v>162</v>
-      </c>
-      <c r="U29" s="117"/>
-      <c r="V29" s="117"/>
+      <c r="P29" s="107" t="s">
+        <v>161</v>
+      </c>
+      <c r="Q29" s="107" t="s">
+        <v>161</v>
+      </c>
+      <c r="R29" s="107" t="s">
+        <v>161</v>
+      </c>
+      <c r="S29" s="107" t="s">
+        <v>161</v>
+      </c>
+      <c r="T29" s="107" t="s">
+        <v>161</v>
+      </c>
+      <c r="U29" s="107"/>
+      <c r="V29" s="107"/>
       <c r="W29" s="88" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="X29" s="89"/>
       <c r="Y29" s="15"/>
@@ -4187,26 +4195,26 @@
       <c r="J30" s="7"/>
       <c r="K30" s="7"/>
       <c r="L30" s="7"/>
-      <c r="M30" s="122" t="s">
-        <v>157</v>
-      </c>
-      <c r="N30" s="123"/>
-      <c r="O30" s="123"/>
-      <c r="P30" s="123"/>
-      <c r="Q30" s="123"/>
-      <c r="R30" s="124">
+      <c r="M30" s="141" t="s">
+        <v>156</v>
+      </c>
+      <c r="N30" s="142"/>
+      <c r="O30" s="142"/>
+      <c r="P30" s="142"/>
+      <c r="Q30" s="142"/>
+      <c r="R30" s="110">
         <f>SUM(R3:R27)</f>
-        <v>28.2987</v>
-      </c>
-      <c r="S30" s="108"/>
-      <c r="T30" s="125">
+        <v>28.277438</v>
+      </c>
+      <c r="S30" s="100"/>
+      <c r="T30" s="111">
         <f>SUM(T3:T27)</f>
-        <v>13819.096000000003</v>
-      </c>
-      <c r="U30" s="125"/>
-      <c r="V30" s="126">
+        <v>13829.617210000002</v>
+      </c>
+      <c r="U30" s="111"/>
+      <c r="V30" s="112">
         <f>SUM(V3:V27)</f>
-        <v>27340.231000000003</v>
+        <v>27361.578710000005</v>
       </c>
       <c r="W30" s="7"/>
       <c r="X30" s="7"/>
@@ -4223,23 +4231,23 @@
       <c r="J31" s="7"/>
       <c r="K31" s="7"/>
       <c r="L31" s="7"/>
-      <c r="M31" s="127" t="s">
-        <v>158</v>
-      </c>
-      <c r="N31" s="128"/>
-      <c r="O31" s="128"/>
-      <c r="P31" s="128"/>
-      <c r="Q31" s="128"/>
-      <c r="R31" s="111"/>
-      <c r="S31" s="111"/>
-      <c r="T31" s="129">
+      <c r="M31" s="143" t="s">
+        <v>157</v>
+      </c>
+      <c r="N31" s="144"/>
+      <c r="O31" s="144"/>
+      <c r="P31" s="144"/>
+      <c r="Q31" s="144"/>
+      <c r="R31" s="101"/>
+      <c r="S31" s="101"/>
+      <c r="T31" s="113">
         <f>T30/500</f>
-        <v>27.638192000000007</v>
-      </c>
-      <c r="U31" s="129"/>
-      <c r="V31" s="130">
+        <v>27.659234420000004</v>
+      </c>
+      <c r="U31" s="113"/>
+      <c r="V31" s="114">
         <f>V30/1000</f>
-        <v>27.340231000000003</v>
+        <v>27.361578710000007</v>
       </c>
       <c r="W31" s="7"/>
       <c r="X31" s="7"/>
@@ -4249,48 +4257,48 @@
       <c r="A32" s="1"/>
       <c r="D32" s="10"/>
       <c r="E32" s="9"/>
-      <c r="N32" s="118" t="s">
-        <v>190</v>
-      </c>
-      <c r="O32" s="119"/>
-      <c r="P32" s="119"/>
-      <c r="Q32" s="120"/>
-      <c r="R32" s="120">
+      <c r="N32" s="134" t="s">
+        <v>189</v>
+      </c>
+      <c r="O32" s="135"/>
+      <c r="P32" s="135"/>
+      <c r="Q32" s="108"/>
+      <c r="R32" s="108">
         <f>5.45+4.23+1</f>
         <v>10.68</v>
       </c>
-      <c r="S32" s="120"/>
-      <c r="T32" s="120">
+      <c r="S32" s="108"/>
+      <c r="T32" s="108">
         <f>5.45+4.23+1</f>
         <v>10.68</v>
       </c>
-      <c r="U32" s="120"/>
-      <c r="V32" s="121"/>
+      <c r="U32" s="108"/>
+      <c r="V32" s="109"/>
       <c r="X32" s="15"/>
       <c r="Y32" s="15"/>
     </row>
     <row r="33" spans="1:25" ht="16.5" thickBot="1">
       <c r="A33" s="1"/>
       <c r="D33" s="9"/>
-      <c r="N33" s="109" t="s">
-        <v>191</v>
-      </c>
-      <c r="O33" s="110"/>
-      <c r="P33" s="110"/>
-      <c r="Q33" s="111"/>
-      <c r="R33" s="112">
+      <c r="N33" s="136" t="s">
+        <v>190</v>
+      </c>
+      <c r="O33" s="137"/>
+      <c r="P33" s="137"/>
+      <c r="Q33" s="101"/>
+      <c r="R33" s="102">
         <f>R32+R30</f>
-        <v>38.978700000000003</v>
-      </c>
-      <c r="S33" s="111"/>
-      <c r="T33" s="113">
+        <v>38.957437999999996</v>
+      </c>
+      <c r="S33" s="101"/>
+      <c r="T33" s="103">
         <f>T32+T30</f>
-        <v>13829.776000000003</v>
-      </c>
-      <c r="U33" s="111"/>
-      <c r="V33" s="114">
+        <v>13840.297210000002</v>
+      </c>
+      <c r="U33" s="101"/>
+      <c r="V33" s="104">
         <f>V30+T32</f>
-        <v>27350.911000000004</v>
+        <v>27372.258710000006</v>
       </c>
       <c r="X33" s="15"/>
       <c r="Y33" s="15"/>
@@ -4299,7 +4307,7 @@
       <c r="A34" s="1"/>
       <c r="C34" s="10"/>
       <c r="D34" s="9"/>
-      <c r="N34" s="107"/>
+      <c r="N34" s="99"/>
       <c r="X34" s="15"/>
       <c r="Y34" s="15"/>
     </row>
@@ -4557,29 +4565,29 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="P3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="P4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="P5" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="P8" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="P9" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="P10" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="P11" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="P13" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="P12" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="P14" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="P17" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="P18" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="P20" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="P6" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="P7" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="P21" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="P25" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="P22" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="P15" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="P16" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="P27" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="P23" r:id="rId22" xr:uid="{46B85C4E-4D34-4998-B97F-463A47B0B565}"/>
-    <hyperlink ref="P26" r:id="rId23" xr:uid="{4EB02A88-D6E7-49CF-AD1C-AD4BFE76142C}"/>
+    <hyperlink ref="P3" r:id="rId1"/>
+    <hyperlink ref="P4" r:id="rId2"/>
+    <hyperlink ref="P5" r:id="rId3"/>
+    <hyperlink ref="P8" r:id="rId4"/>
+    <hyperlink ref="P9" r:id="rId5"/>
+    <hyperlink ref="P10" r:id="rId6"/>
+    <hyperlink ref="P11" r:id="rId7"/>
+    <hyperlink ref="P13" r:id="rId8"/>
+    <hyperlink ref="P12" r:id="rId9"/>
+    <hyperlink ref="P14" r:id="rId10"/>
+    <hyperlink ref="P17" r:id="rId11"/>
+    <hyperlink ref="P18" r:id="rId12"/>
+    <hyperlink ref="P6" r:id="rId13"/>
+    <hyperlink ref="P7" r:id="rId14"/>
+    <hyperlink ref="P21" r:id="rId15"/>
+    <hyperlink ref="P25" r:id="rId16"/>
+    <hyperlink ref="P22" r:id="rId17"/>
+    <hyperlink ref="P15" r:id="rId18"/>
+    <hyperlink ref="P16" r:id="rId19"/>
+    <hyperlink ref="P27" r:id="rId20"/>
+    <hyperlink ref="P23" r:id="rId21"/>
+    <hyperlink ref="P26" r:id="rId22"/>
+    <hyperlink ref="P20" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId24"/>

</xml_diff>

<commit_message>
Interface BOM reviewed and aliexpress shipping cost corrected in both BOMs.
</commit_message>
<xml_diff>
--- a/Deliverables/Control_Board/BOM/LCSC_CB_ 500.xlsx
+++ b/Deliverables/Control_Board/BOM/LCSC_CB_ 500.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24701"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\ChrisitanRaun-AnnanasMotor\Deliverables\Control_Board\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\ChrisitanRaun-AnnanasMotor\Deliverables\Control_Board\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4181602-BF45-49AD-B335-A5CDF466C7F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -624,7 +625,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00000"/>
@@ -1709,6 +1710,15 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1755,15 +1765,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2041,7 +2042,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Y46"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
@@ -2071,32 +2072,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25" ht="16.5" thickBot="1">
-      <c r="A1" s="138" t="s">
+      <c r="A1" s="141" t="s">
         <v>165</v>
       </c>
-      <c r="B1" s="139"/>
-      <c r="C1" s="139"/>
-      <c r="D1" s="139"/>
-      <c r="E1" s="139"/>
-      <c r="F1" s="139"/>
-      <c r="G1" s="139"/>
-      <c r="H1" s="139"/>
-      <c r="I1" s="139"/>
-      <c r="J1" s="139"/>
-      <c r="K1" s="139"/>
-      <c r="L1" s="139"/>
-      <c r="M1" s="139"/>
-      <c r="N1" s="139"/>
-      <c r="O1" s="139"/>
-      <c r="P1" s="139"/>
-      <c r="Q1" s="139"/>
-      <c r="R1" s="139"/>
-      <c r="S1" s="139"/>
-      <c r="T1" s="139"/>
-      <c r="U1" s="139"/>
-      <c r="V1" s="139"/>
-      <c r="W1" s="139"/>
-      <c r="X1" s="140"/>
+      <c r="B1" s="142"/>
+      <c r="C1" s="142"/>
+      <c r="D1" s="142"/>
+      <c r="E1" s="142"/>
+      <c r="F1" s="142"/>
+      <c r="G1" s="142"/>
+      <c r="H1" s="142"/>
+      <c r="I1" s="142"/>
+      <c r="J1" s="142"/>
+      <c r="K1" s="142"/>
+      <c r="L1" s="142"/>
+      <c r="M1" s="142"/>
+      <c r="N1" s="142"/>
+      <c r="O1" s="142"/>
+      <c r="P1" s="142"/>
+      <c r="Q1" s="142"/>
+      <c r="R1" s="142"/>
+      <c r="S1" s="142"/>
+      <c r="T1" s="142"/>
+      <c r="U1" s="142"/>
+      <c r="V1" s="142"/>
+      <c r="W1" s="142"/>
+      <c r="X1" s="143"/>
     </row>
     <row r="2" spans="1:25" ht="16.5" thickBot="1">
       <c r="A2" s="3" t="s">
@@ -2176,7 +2177,7 @@
       <c r="A3" s="6">
         <v>1</v>
       </c>
-      <c r="B3" s="145" t="s">
+      <c r="B3" s="148" t="s">
         <v>15</v>
       </c>
       <c r="C3" s="29" t="s">
@@ -2240,7 +2241,7 @@
       <c r="U3" s="35">
         <v>6.8199999999999997E-2</v>
       </c>
-      <c r="V3" s="151">
+      <c r="V3" s="135">
         <f>U3*K3</f>
         <v>276.20999999999998</v>
       </c>
@@ -2251,7 +2252,7 @@
       <c r="A4" s="6">
         <v>2</v>
       </c>
-      <c r="B4" s="146"/>
+      <c r="B4" s="149"/>
       <c r="C4" s="38" t="s">
         <v>25</v>
       </c>
@@ -2324,7 +2325,7 @@
       <c r="A5" s="6">
         <v>3</v>
       </c>
-      <c r="B5" s="146"/>
+      <c r="B5" s="149"/>
       <c r="C5" s="38" t="s">
         <v>31</v>
       </c>
@@ -2398,7 +2399,7 @@
       <c r="A6" s="6">
         <v>4</v>
       </c>
-      <c r="B6" s="146"/>
+      <c r="B6" s="149"/>
       <c r="C6" s="38" t="s">
         <v>37</v>
       </c>
@@ -2472,7 +2473,7 @@
       <c r="A7" s="6">
         <v>5</v>
       </c>
-      <c r="B7" s="147"/>
+      <c r="B7" s="150"/>
       <c r="C7" s="48" t="s">
         <v>44</v>
       </c>
@@ -2506,11 +2507,11 @@
       <c r="M7" s="53">
         <v>4</v>
       </c>
-      <c r="N7" s="150">
+      <c r="N7" s="134">
         <f t="shared" si="4"/>
         <v>2000</v>
       </c>
-      <c r="O7" s="150">
+      <c r="O7" s="134">
         <f t="shared" si="1"/>
         <v>4000</v>
       </c>
@@ -2534,7 +2535,7 @@
       <c r="U7" s="56">
         <v>1.8E-3</v>
       </c>
-      <c r="V7" s="152">
+      <c r="V7" s="136">
         <f t="shared" si="3"/>
         <v>7.38</v>
       </c>
@@ -2622,7 +2623,7 @@
       <c r="A9" s="6">
         <v>7</v>
       </c>
-      <c r="B9" s="145" t="s">
+      <c r="B9" s="148" t="s">
         <v>59</v>
       </c>
       <c r="C9" s="29" t="s">
@@ -2698,7 +2699,7 @@
       <c r="A10" s="6">
         <v>8</v>
       </c>
-      <c r="B10" s="147"/>
+      <c r="B10" s="150"/>
       <c r="C10" s="48" t="s">
         <v>66</v>
       </c>
@@ -2772,7 +2773,7 @@
       <c r="A11" s="6">
         <v>9</v>
       </c>
-      <c r="B11" s="145" t="s">
+      <c r="B11" s="148" t="s">
         <v>72</v>
       </c>
       <c r="C11" s="29" t="s">
@@ -2836,7 +2837,7 @@
       <c r="U11" s="35">
         <v>8.9999999999999998E-4</v>
       </c>
-      <c r="V11" s="151">
+      <c r="V11" s="135">
         <f t="shared" si="3"/>
         <v>10.89</v>
       </c>
@@ -2848,7 +2849,7 @@
       <c r="A12" s="6">
         <v>10</v>
       </c>
-      <c r="B12" s="146"/>
+      <c r="B12" s="149"/>
       <c r="C12" s="38" t="s">
         <v>79</v>
       </c>
@@ -2922,7 +2923,7 @@
       <c r="A13" s="6">
         <v>11</v>
       </c>
-      <c r="B13" s="146"/>
+      <c r="B13" s="149"/>
       <c r="C13" s="38" t="s">
         <v>84</v>
       </c>
@@ -2996,7 +2997,7 @@
       <c r="A14" s="6">
         <v>12</v>
       </c>
-      <c r="B14" s="146"/>
+      <c r="B14" s="149"/>
       <c r="C14" s="38" t="s">
         <v>89</v>
       </c>
@@ -3070,7 +3071,7 @@
       <c r="A15" s="6">
         <v>13</v>
       </c>
-      <c r="B15" s="148"/>
+      <c r="B15" s="151"/>
       <c r="C15" s="92" t="s">
         <v>94</v>
       </c>
@@ -3144,7 +3145,7 @@
       <c r="A16" s="6">
         <v>14</v>
       </c>
-      <c r="B16" s="148"/>
+      <c r="B16" s="151"/>
       <c r="C16" s="92" t="s">
         <v>99</v>
       </c>
@@ -3218,7 +3219,7 @@
       <c r="A17" s="6">
         <v>15</v>
       </c>
-      <c r="B17" s="147"/>
+      <c r="B17" s="150"/>
       <c r="C17" s="48" t="s">
         <v>104</v>
       </c>
@@ -3252,11 +3253,11 @@
       <c r="M17" s="53">
         <v>1</v>
       </c>
-      <c r="N17" s="150">
+      <c r="N17" s="134">
         <f t="shared" si="4"/>
         <v>500</v>
       </c>
-      <c r="O17" s="150">
+      <c r="O17" s="134">
         <f t="shared" si="1"/>
         <v>1000</v>
       </c>
@@ -3280,7 +3281,7 @@
       <c r="U17" s="56">
         <v>0.01</v>
       </c>
-      <c r="V17" s="152">
+      <c r="V17" s="136">
         <f t="shared" si="3"/>
         <v>10.4</v>
       </c>
@@ -3368,7 +3369,7 @@
       <c r="A19" s="6">
         <v>17</v>
       </c>
-      <c r="B19" s="145" t="s">
+      <c r="B19" s="148" t="s">
         <v>116</v>
       </c>
       <c r="C19" s="29" t="s">
@@ -3432,7 +3433,7 @@
       <c r="U19" s="119">
         <v>21.26</v>
       </c>
-      <c r="V19" s="151">
+      <c r="V19" s="135">
         <f t="shared" si="3"/>
         <v>21472.600000000002</v>
       </c>
@@ -3444,7 +3445,7 @@
       <c r="A20" s="6">
         <v>18</v>
       </c>
-      <c r="B20" s="146"/>
+      <c r="B20" s="149"/>
       <c r="C20" s="80" t="s">
         <v>120</v>
       </c>
@@ -3518,7 +3519,7 @@
       <c r="A21" s="6">
         <v>19</v>
       </c>
-      <c r="B21" s="146"/>
+      <c r="B21" s="149"/>
       <c r="C21" s="38" t="s">
         <v>125</v>
       </c>
@@ -3596,7 +3597,7 @@
       <c r="A22" s="6">
         <v>20</v>
       </c>
-      <c r="B22" s="147"/>
+      <c r="B22" s="150"/>
       <c r="C22" s="48" t="s">
         <v>129</v>
       </c>
@@ -3630,11 +3631,11 @@
       <c r="M22" s="97">
         <v>1</v>
       </c>
-      <c r="N22" s="150">
+      <c r="N22" s="134">
         <f t="shared" si="4"/>
         <v>500</v>
       </c>
-      <c r="O22" s="150">
+      <c r="O22" s="134">
         <f t="shared" si="1"/>
         <v>1000</v>
       </c>
@@ -3658,7 +3659,7 @@
       <c r="U22" s="56">
         <v>0.4</v>
       </c>
-      <c r="V22" s="152">
+      <c r="V22" s="136">
         <f t="shared" si="3"/>
         <v>404</v>
       </c>
@@ -3674,7 +3675,7 @@
       <c r="A23" s="6">
         <v>21</v>
       </c>
-      <c r="B23" s="145" t="s">
+      <c r="B23" s="148" t="s">
         <v>135</v>
       </c>
       <c r="C23" s="29" t="s">
@@ -3750,7 +3751,7 @@
       <c r="A24" s="6">
         <v>22</v>
       </c>
-      <c r="B24" s="147"/>
+      <c r="B24" s="150"/>
       <c r="C24" s="48" t="s">
         <v>139</v>
       </c>
@@ -3824,7 +3825,7 @@
       <c r="A25" s="6">
         <v>23</v>
       </c>
-      <c r="B25" s="149" t="s">
+      <c r="B25" s="152" t="s">
         <v>143</v>
       </c>
       <c r="C25" s="116" t="s">
@@ -3887,7 +3888,7 @@
       <c r="U25" s="35">
         <v>0.48</v>
       </c>
-      <c r="V25" s="151">
+      <c r="V25" s="135">
         <f t="shared" si="3"/>
         <v>67.2</v>
       </c>
@@ -3901,7 +3902,7 @@
       <c r="A26" s="6">
         <v>24</v>
       </c>
-      <c r="B26" s="149"/>
+      <c r="B26" s="152"/>
       <c r="C26" s="38" t="s">
         <v>170</v>
       </c>
@@ -3974,7 +3975,7 @@
       <c r="A27" s="6">
         <v>25</v>
       </c>
-      <c r="B27" s="146"/>
+      <c r="B27" s="149"/>
       <c r="C27" s="38" t="s">
         <v>176</v>
       </c>
@@ -4036,7 +4037,7 @@
       <c r="U27" s="43">
         <v>0.45</v>
       </c>
-      <c r="V27" s="152">
+      <c r="V27" s="136">
         <f>U27*K27</f>
         <v>459</v>
       </c>
@@ -4050,7 +4051,7 @@
       <c r="A28" s="6">
         <v>26</v>
       </c>
-      <c r="B28" s="146"/>
+      <c r="B28" s="149"/>
       <c r="C28" s="81" t="s">
         <v>149</v>
       </c>
@@ -4119,7 +4120,7 @@
       <c r="A29" s="98">
         <v>27</v>
       </c>
-      <c r="B29" s="147"/>
+      <c r="B29" s="150"/>
       <c r="C29" s="86" t="s">
         <v>153</v>
       </c>
@@ -4195,13 +4196,13 @@
       <c r="J30" s="7"/>
       <c r="K30" s="7"/>
       <c r="L30" s="7"/>
-      <c r="M30" s="141" t="s">
+      <c r="M30" s="144" t="s">
         <v>156</v>
       </c>
-      <c r="N30" s="142"/>
-      <c r="O30" s="142"/>
-      <c r="P30" s="142"/>
-      <c r="Q30" s="142"/>
+      <c r="N30" s="145"/>
+      <c r="O30" s="145"/>
+      <c r="P30" s="145"/>
+      <c r="Q30" s="145"/>
       <c r="R30" s="110">
         <f>SUM(R3:R27)</f>
         <v>28.277438</v>
@@ -4231,13 +4232,13 @@
       <c r="J31" s="7"/>
       <c r="K31" s="7"/>
       <c r="L31" s="7"/>
-      <c r="M31" s="143" t="s">
+      <c r="M31" s="146" t="s">
         <v>157</v>
       </c>
-      <c r="N31" s="144"/>
-      <c r="O31" s="144"/>
-      <c r="P31" s="144"/>
-      <c r="Q31" s="144"/>
+      <c r="N31" s="147"/>
+      <c r="O31" s="147"/>
+      <c r="P31" s="147"/>
+      <c r="Q31" s="147"/>
       <c r="R31" s="101"/>
       <c r="S31" s="101"/>
       <c r="T31" s="113">
@@ -4257,48 +4258,45 @@
       <c r="A32" s="1"/>
       <c r="D32" s="10"/>
       <c r="E32" s="9"/>
-      <c r="N32" s="134" t="s">
+      <c r="N32" s="137" t="s">
         <v>189</v>
       </c>
-      <c r="O32" s="135"/>
-      <c r="P32" s="135"/>
+      <c r="O32" s="138"/>
+      <c r="P32" s="138"/>
       <c r="Q32" s="108"/>
-      <c r="R32" s="108">
-        <f>5.45+4.23+1</f>
-        <v>10.68</v>
-      </c>
+      <c r="R32" s="108"/>
       <c r="S32" s="108"/>
       <c r="T32" s="108">
-        <f>5.45+4.23+1</f>
-        <v>10.68</v>
+        <f>50.2+154.78+11.19</f>
+        <v>216.17000000000002</v>
       </c>
       <c r="U32" s="108"/>
-      <c r="V32" s="109"/>
+      <c r="V32" s="109">
+        <f>133.4+50.2+19.44</f>
+        <v>203.04000000000002</v>
+      </c>
       <c r="X32" s="15"/>
       <c r="Y32" s="15"/>
     </row>
     <row r="33" spans="1:25" ht="16.5" thickBot="1">
       <c r="A33" s="1"/>
       <c r="D33" s="9"/>
-      <c r="N33" s="136" t="s">
+      <c r="N33" s="139" t="s">
         <v>190</v>
       </c>
-      <c r="O33" s="137"/>
-      <c r="P33" s="137"/>
+      <c r="O33" s="140"/>
+      <c r="P33" s="140"/>
       <c r="Q33" s="101"/>
-      <c r="R33" s="102">
-        <f>R32+R30</f>
-        <v>38.957437999999996</v>
-      </c>
+      <c r="R33" s="102"/>
       <c r="S33" s="101"/>
       <c r="T33" s="103">
         <f>T32+T30</f>
-        <v>13840.297210000002</v>
+        <v>14045.787210000002</v>
       </c>
       <c r="U33" s="101"/>
       <c r="V33" s="104">
         <f>V30+T32</f>
-        <v>27372.258710000006</v>
+        <v>27577.748710000003</v>
       </c>
       <c r="X33" s="15"/>
       <c r="Y33" s="15"/>
@@ -4565,29 +4563,29 @@
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="P3" r:id="rId1"/>
-    <hyperlink ref="P4" r:id="rId2"/>
-    <hyperlink ref="P5" r:id="rId3"/>
-    <hyperlink ref="P8" r:id="rId4"/>
-    <hyperlink ref="P9" r:id="rId5"/>
-    <hyperlink ref="P10" r:id="rId6"/>
-    <hyperlink ref="P11" r:id="rId7"/>
-    <hyperlink ref="P13" r:id="rId8"/>
-    <hyperlink ref="P12" r:id="rId9"/>
-    <hyperlink ref="P14" r:id="rId10"/>
-    <hyperlink ref="P17" r:id="rId11"/>
-    <hyperlink ref="P18" r:id="rId12"/>
-    <hyperlink ref="P6" r:id="rId13"/>
-    <hyperlink ref="P7" r:id="rId14"/>
-    <hyperlink ref="P21" r:id="rId15"/>
-    <hyperlink ref="P25" r:id="rId16"/>
-    <hyperlink ref="P22" r:id="rId17"/>
-    <hyperlink ref="P15" r:id="rId18"/>
-    <hyperlink ref="P16" r:id="rId19"/>
-    <hyperlink ref="P27" r:id="rId20"/>
-    <hyperlink ref="P23" r:id="rId21"/>
-    <hyperlink ref="P26" r:id="rId22"/>
-    <hyperlink ref="P20" r:id="rId23"/>
+    <hyperlink ref="P3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="P4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="P5" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="P8" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="P9" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="P10" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="P11" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="P13" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="P12" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="P14" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="P17" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="P18" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="P6" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="P7" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="P21" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="P25" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="P22" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="P15" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="P16" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="P27" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="P23" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="P26" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="P20" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId24"/>

</xml_diff>